<commit_message>
Calendar redesign + commission fix: Básico now pays commission
Calendar page redesign:
- New hero with gradient (blue→cyan→purple)
- Stats grid (hoy, semana, sin confirmar, atendidas)
- Container with gradient accent bar
- Styled FullCalendar buttons with gradient + shadows
- Legend below calendar explaining color codes
- Fixed double-render by removing header widget (now rendered inline)

Commission fix:
- COMMISSIONABLE_PLANS now includes 'basico' (Free remains excluded)
- halfAmount uses 1.5x multiplier divided by 2 (was 3x/2)
- Básico $299 → $448.50 commission ($224.25 x 2 payments)
- Pro $599 → $898.50 ($449.25 x 2)
- Clínica $1199 → $1798.50 ($899.25 x 2)

Regenerated docs:
- docs/sales-cashflow.xlsx
- docs/acuerdo-vendedor.xlsx
- docs/DocFacil-Kit-Vendedor-2026.xlsx
All with new commission rules + Básico as qualifying plan.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DocFacil-Kit-Vendedor-2026.xlsx
+++ b/docs/DocFacil-Kit-Vendedor-2026.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="296">
   <si>
     <t>DocFácil — Kit de Vendedor 2026</t>
   </si>
@@ -119,7 +119,7 @@
     <t>—</t>
   </si>
   <si>
-    <t>Doctores curiosos. Gancho para conversión.</t>
+    <t>Doctores curiosos. Sin comisión. Gancho para conversión.</t>
   </si>
   <si>
     <t>BÁSICO</t>
@@ -131,7 +131,7 @@
     <t>$149 (50% off)</t>
   </si>
   <si>
-    <t>Doctores individuales que buscan eficiencia básica.</t>
+    <t>Doctores individuales. Comisión: $448.50 por venta.</t>
   </si>
   <si>
     <t>PRO ⭐</t>
@@ -146,7 +146,7 @@
     <t>Ilimitados</t>
   </si>
   <si>
-    <t>EL QUE MÁS VENDE. Incluye TODA la IA.</t>
+    <t>EL QUE MÁS VENDE. TODA la IA. Comisión: $898.50 por venta.</t>
   </si>
   <si>
     <t>CLÍNICA</t>
@@ -158,10 +158,10 @@
     <t>$599 (50% off)</t>
   </si>
   <si>
-    <t>Clínicas con 4+ doctores. Multi-sucursal.</t>
-  </si>
-  <si>
-    <t>⚠️ IMPORTANTE: Las comisiones solo se pagan por planes PRO y CLÍNICA (NO Free ni Básico)</t>
+    <t>Clínicas grandes. Comisión: $1,798.50 por venta.</t>
+  </si>
+  <si>
+    <t>✅ TODOS los planes de pago (Básico, Pro y Clínica) pagan comisión. Solo el plan Free NO.</t>
   </si>
   <si>
     <t>✨ FEATURES INCLUIDAS POR PLAN</t>
@@ -686,6 +686,12 @@
     <t>Básico</t>
   </si>
   <si>
+    <t>$448.50</t>
+  </si>
+  <si>
+    <t>$224.25 + $224.25</t>
+  </si>
+  <si>
     <t>Pro ⭐</t>
   </si>
   <si>
@@ -722,13 +728,13 @@
     <t>Starter</t>
   </si>
   <si>
-    <t>3 Pro</t>
-  </si>
-  <si>
-    <t>3 x $898</t>
-  </si>
-  <si>
-    <t>$2,695</t>
+    <t>3 Básico + 2 Pro</t>
+  </si>
+  <si>
+    <t>3x$448.50 + 2x$898.50</t>
+  </si>
+  <si>
+    <t>$3,142.50</t>
   </si>
   <si>
     <t>Medium</t>
@@ -737,10 +743,10 @@
     <t>5 Pro + 1 Clínica</t>
   </si>
   <si>
-    <t>5x$898 + 1x$1,798</t>
-  </si>
-  <si>
-    <t>$6,290</t>
+    <t>5x$898.50 + 1x$1,798.50</t>
+  </si>
+  <si>
+    <t>$6,291</t>
   </si>
   <si>
     <t>Top</t>
@@ -749,10 +755,22 @@
     <t>10 Pro + 2 Clínica</t>
   </si>
   <si>
-    <t>10x$898 + 2x$1,798</t>
-  </si>
-  <si>
-    <t>$12,580</t>
+    <t>10x$898.50 + 2x$1,798.50</t>
+  </si>
+  <si>
+    <t>$12,582</t>
+  </si>
+  <si>
+    <t>Elite</t>
+  </si>
+  <si>
+    <t>5 Básico + 10 Pro + 3 Clínica</t>
+  </si>
+  <si>
+    <t>Mix completo</t>
+  </si>
+  <si>
+    <t>$16,618.50</t>
   </si>
   <si>
     <t>🔗 LINKS IMPORTANTES</t>
@@ -983,7 +1001,7 @@
       <strike val="0"/>
       <u val="none"/>
       <sz val="12"/>
-      <color rgb="FFDC2626"/>
+      <color rgb="FF065F46"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -1113,7 +1131,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEE2E2"/>
+        <fgColor rgb="FFD1FAE5"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -1694,161 +1712,161 @@
   <sheetData>
     <row r="1" spans="1:3" customHeight="1" ht="40">
       <c r="A1" s="5" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" spans="1:3" customHeight="1" ht="25">
       <c r="A3" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B3" s="40" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:3" customHeight="1" ht="25">
       <c r="A4" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B4" s="40" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" spans="1:3" customHeight="1" ht="25">
       <c r="A5" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B5" s="40" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:3" customHeight="1" ht="25">
       <c r="A6" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B6" s="40" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7" spans="1:3" customHeight="1" ht="25">
       <c r="A7" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" spans="1:3" customHeight="1" ht="25">
       <c r="A8" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B8" s="40" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" spans="1:3" customHeight="1" ht="25">
       <c r="A9" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B9" s="40" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10" spans="1:3" customHeight="1" ht="25">
       <c r="A10" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B10" s="40" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
     <row r="11" spans="1:3" customHeight="1" ht="25">
       <c r="A11" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B11" s="40" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
     </row>
     <row r="12" spans="1:3" customHeight="1" ht="25">
       <c r="A12" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
     </row>
     <row r="13" spans="1:3" customHeight="1" ht="25">
       <c r="A13" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B13" s="40" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
     </row>
     <row r="14" spans="1:3" customHeight="1" ht="25">
       <c r="A14" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B14" s="40" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="15" spans="1:3" customHeight="1" ht="25">
       <c r="A15" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B15" s="40" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
     </row>
     <row r="16" spans="1:3" customHeight="1" ht="25">
       <c r="A16" s="39" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B16" s="40" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -3261,7 +3279,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="true" style="0"/>
@@ -3321,99 +3339,113 @@
         <v>33</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>29</v>
+        <v>220</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="19" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B9" s="19" t="s">
         <v>37</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="19" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>42</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="35" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="36" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B15" s="36" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C15" s="36" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D15" s="36" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="12" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="12" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="12" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>242</v>
+        <v>244</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -3443,71 +3475,71 @@
   <sheetData>
     <row r="1" spans="1:2" customHeight="1" ht="40">
       <c r="A1" s="5" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:2" customHeight="1" ht="25">
       <c r="A3" s="37" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="B3" s="38" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:2" customHeight="1" ht="25">
       <c r="A4" s="37" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" spans="1:2" customHeight="1" ht="25">
       <c r="A5" s="37" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" spans="1:2" customHeight="1" ht="25">
       <c r="A6" s="37" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7" spans="1:2" customHeight="1" ht="25">
       <c r="A7" s="37" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8" spans="1:2" customHeight="1" ht="25">
       <c r="A8" s="37" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
     </row>
     <row r="9" spans="1:2" customHeight="1" ht="25">
       <c r="A9" s="37" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:2" customHeight="1" ht="25">
       <c r="A10" s="37" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corregir comisión a 3× en todo: código, guía ventas, docs, xlsx
El multiplicador correcto es 3× la mensualidad, no 1.5×.

- Commission::halfAmount() → 1.5× por mitad (3× total / 2)
- Guía de venta: Básico $447, Pro $897, Clínica $1,497
- docs/generate-vendedor-acuerdo.php: tabla, calculadora, ejemplos
- docs/generate-vendedor-kit.php: comisiones, metas mensuales
- docs/generate-cashflow.php: multiplier 3 en los 3 planes
- CLAUDE.md: actualizado
- 3 xlsx regenerados

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DocFacil-Kit-Vendedor-2026.xlsx
+++ b/docs/DocFacil-Kit-Vendedor-2026.xlsx
@@ -124,7 +124,7 @@
     <t>$74 (50% off)</t>
   </si>
   <si>
-    <t>Doctores individuales. Comisión: $223.50 por venta.</t>
+    <t>Doctores individuales. Comisión: $447 por venta.</t>
   </si>
   <si>
     <t>PRO ⭐</t>
@@ -139,7 +139,7 @@
     <t>Ilimitados</t>
   </si>
   <si>
-    <t>EL QUE MÁS VENDE. Odontograma + Portal + Multi-doctor. Comisión: $448.50 por venta.</t>
+    <t>EL QUE MÁS VENDE. Odontograma + Portal + Multi-doctor. Comisión: $897 por venta.</t>
   </si>
   <si>
     <t>CLÍNICA</t>
@@ -151,7 +151,7 @@
     <t>$249 (50% off)</t>
   </si>
   <si>
-    <t>Clínicas grandes. Comisión: $748.50 por venta.</t>
+    <t>Clínicas grandes. Comisión: $1,497 por venta.</t>
   </si>
   <si>
     <t>✅ TODOS los planes de pago (Básico, Pro y Clínica) pagan comisión. Solo el plan Free NO.</t>
@@ -484,7 +484,7 @@
     <t>💰 ESQUEMA DE COMISIONES</t>
   </si>
   <si>
-    <t>🎯 GANAS 1.5 MENSUALIDADES POR CADA CLIENTE DE PAGO (Básico, Pro o Clínica)</t>
+    <t>🎯 GANAS 3 MENSUALIDADES POR CADA CLIENTE DE PAGO (Básico, Pro o Clínica)</t>
   </si>
   <si>
     <t>Se paga 50% con el primer pago del cliente, 50% con el segundo pago</t>
@@ -493,7 +493,7 @@
     <t>Precio cliente/mes</t>
   </si>
   <si>
-    <t>Comisión total (1.5x)</t>
+    <t>Comisión total (3x)</t>
   </si>
   <si>
     <t>½ primer pago + ½ segundo pago</t>
@@ -505,28 +505,28 @@
     <t>Básico</t>
   </si>
   <si>
-    <t>$223.50</t>
-  </si>
-  <si>
-    <t>$111.75 + $111.75</t>
+    <t>$447</t>
+  </si>
+  <si>
+    <t>$223.50 + $223.50</t>
   </si>
   <si>
     <t>Pro ⭐</t>
   </si>
   <si>
-    <t>$448.50</t>
-  </si>
-  <si>
-    <t>$224.25 + $224.25</t>
+    <t>$897</t>
+  </si>
+  <si>
+    <t>$448.50 + $448.50</t>
   </si>
   <si>
     <t>Clínica</t>
   </si>
   <si>
-    <t>$748.50</t>
-  </si>
-  <si>
-    <t>$374.25 + $374.25</t>
+    <t>$1,497</t>
+  </si>
+  <si>
+    <t>$748.50 + $748.50</t>
   </si>
   <si>
     <t>📊 METAS MENSUALES PARA VENDEDOR</t>
@@ -550,10 +550,10 @@
     <t>3 Básico + 2 Pro</t>
   </si>
   <si>
-    <t>3x$223.50 + 2x$448.50</t>
-  </si>
-  <si>
-    <t>$1,567.50</t>
+    <t>3x$447 + 2x$897</t>
+  </si>
+  <si>
+    <t>$3,135</t>
   </si>
   <si>
     <t>Medium</t>
@@ -562,10 +562,10 @@
     <t>5 Pro + 1 Clínica</t>
   </si>
   <si>
-    <t>5x$448.50 + 1x$748.50</t>
-  </si>
-  <si>
-    <t>$2,991</t>
+    <t>5x$897 + 1x$1,497</t>
+  </si>
+  <si>
+    <t>$5,982</t>
   </si>
   <si>
     <t>Top</t>
@@ -574,10 +574,10 @@
     <t>10 Pro + 2 Clínica</t>
   </si>
   <si>
-    <t>10x$448.50 + 2x$748.50</t>
-  </si>
-  <si>
-    <t>$5,982</t>
+    <t>10x$897 + 2x$1,497</t>
+  </si>
+  <si>
+    <t>$11,964</t>
   </si>
   <si>
     <t>Elite</t>

</xml_diff>